<commit_message>
feat(products): importar decants desde columnas variacion N del Excel
El importador lee 'variacion 1..3' + 'precio variacion 1..3' y los envia
como variants[] al bulk-import; la vista previa muestra los decants de
cada fila. Plantilla y ejemplo regenerados con las 6 columnas nuevas.
</commit_message>
<xml_diff>
--- a/public/ejemplo-importacion-productos.xlsx
+++ b/public/ejemplo-importacion-productos.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AG4"/>
+  <dimension ref="A1:AM4"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -434,6 +434,12 @@
     <col min="31" max="31" width="22.83203125" customWidth="1"/>
     <col min="32" max="32" width="22.83203125" customWidth="1"/>
     <col min="33" max="33" width="22.83203125" customWidth="1"/>
+    <col min="34" max="34" width="22.83203125" customWidth="1"/>
+    <col min="35" max="35" width="22.83203125" customWidth="1"/>
+    <col min="36" max="36" width="22.83203125" customWidth="1"/>
+    <col min="37" max="37" width="22.83203125" customWidth="1"/>
+    <col min="38" max="38" width="22.83203125" customWidth="1"/>
+    <col min="39" max="39" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -536,6 +542,24 @@
       <c r="AG1" t="str">
         <v>descripcion_firma</v>
       </c>
+      <c r="AH1" t="str">
+        <v>variacion 1</v>
+      </c>
+      <c r="AI1" t="str">
+        <v>precio variacion 1</v>
+      </c>
+      <c r="AJ1" t="str">
+        <v>variacion 2</v>
+      </c>
+      <c r="AK1" t="str">
+        <v>precio variacion 2</v>
+      </c>
+      <c r="AL1" t="str">
+        <v>variacion 3</v>
+      </c>
+      <c r="AM1" t="str">
+        <v>precio variacion 3</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -637,6 +661,24 @@
       <c r="AG2" t="str">
         <v>Un equilibrio impecable entre frescura y calidez: el sello inconfundible de Parfums de Marly.</v>
       </c>
+      <c r="AH2">
+        <v>3</v>
+      </c>
+      <c r="AI2">
+        <v>12.5</v>
+      </c>
+      <c r="AJ2">
+        <v>5</v>
+      </c>
+      <c r="AK2">
+        <v>19.5</v>
+      </c>
+      <c r="AL2">
+        <v>10</v>
+      </c>
+      <c r="AM2">
+        <v>34.5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -738,6 +780,24 @@
       <c r="AG3" t="str">
         <v/>
       </c>
+      <c r="AH3">
+        <v>3</v>
+      </c>
+      <c r="AI3">
+        <v>5.5</v>
+      </c>
+      <c r="AJ3">
+        <v>5</v>
+      </c>
+      <c r="AK3">
+        <v>8.5</v>
+      </c>
+      <c r="AL3" t="str">
+        <v/>
+      </c>
+      <c r="AM3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -842,14 +902,14 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AG4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AM4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D38"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1361,9 +1421,37 @@
         <v>Descripción de la firma. La imagen se sube después en el admin</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>variacion 1 · 2 · 3</v>
+      </c>
+      <c r="B37" t="str">
+        <v>número (ml)</v>
+      </c>
+      <c r="C37" t="str">
+        <v>no</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Ml del decant (3, 5, 10…). Hasta 3 decants por producto. La botella completa se crea sola con precio/total_ml</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>precio variacion 1 · 2 · 3</v>
+      </c>
+      <c r="B38" t="str">
+        <v>número</v>
+      </c>
+      <c r="C38" t="str">
+        <v>no</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Precio del decant correspondiente. Si pones el ml, el precio es obligatorio para que se cree</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D38"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: importacion Excel con variantes color x talla + campos editoriales + render.yaml
- Parser extraido a utils/parseProductsExcel.ts (testeable)
- Nuevas columnas: color_hex_N, talla_N, usos_comunes, tallas, combina_con, instagram
- 15 tests vitest incl. round-trip con la plantilla real de public/
- Plantillas regeneradas con el nuevo formato y hoja de ayuda
- Export backup usa las mismas columnas de la plantilla (re-importable)
- Fix TS en FormSectionVariations
- render.yaml: sitio estatico con SPA fallback
</commit_message>
<xml_diff>
--- a/public/ejemplo-importacion-productos.xlsx
+++ b/public/ejemplo-importacion-productos.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,8 +30,11 @@
       <b val="1"/>
       <color rgb="00F5EFC6"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +44,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004D0E12"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006B1A1F"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,9 +64,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:AD3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,12 +451,22 @@
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="25" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
     <col width="15" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
     <col width="15" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="23" max="23"/>
+    <col width="15" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="22" customWidth="1" min="26" max="26"/>
+    <col width="15" customWidth="1" min="27" max="27"/>
+    <col width="15" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
+    <col width="22" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -522,30 +542,80 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>usos_comunes</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>tallas</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>combina_con</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
           <t>variacion_1</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>color_hex_1</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>talla_1</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>precio_variacion_1</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>variacion_2</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>color_hex_2</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>talla_2</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>precio_variacion_2</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>variacion_3</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>color_hex_3</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>talla_3</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>precio_variacion_3</t>
         </is>
@@ -601,27 +671,79 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>39,4 × 30,5 × 19 cm aprox., 6 bolsillos organizadores interiores, compartimento para laptop 15", bolsillo dispensador de toallitas, luggage sleeve</t>
+          <t>Cuero genuino, Hecho a mano en Ecuador, Garantía de por vida</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>Pañalera, Bolso de trabajo, Equipaje de mano</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Mini, Midi, Full</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>https://instagram.com/p/EJEMPLO1|https://res.cloudinary.com/demo/sample.jpg ; https://instagram.com/p/EJEMPLO2</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
           <t>Negro</t>
         </is>
       </c>
-      <c r="P2" t="n">
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>#12100E</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Midi</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
         <v>129</v>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>Espresso</t>
         </is>
       </c>
-      <c r="R2" t="n">
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>#5C3A21</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Midi</t>
+        </is>
+      </c>
+      <c r="Z2" t="n">
         <v>129</v>
       </c>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>#12100E</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="AD2" t="n">
+        <v>139</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -673,31 +795,77 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>33 × 36,8 × 17,8 cm aprox., 6 bolsillos elásticos interiores, 1 bolsillo con cierre, tira con gancho para llaves, cierre magnético</t>
+          <t>Cuero genuino, Interior antimanchas, Correa ajustable</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>Pañalera, Bolso diario</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Única</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>https://instagram.com/p/EJEMPLO3</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
           <t>Beige</t>
         </is>
       </c>
-      <c r="P3" t="n">
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>#D9C7A7</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Única</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
         <v>119</v>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>Espresso</t>
         </is>
       </c>
-      <c r="R3" t="n">
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>#5C3A21</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Única</t>
+        </is>
+      </c>
+      <c r="Z3" t="n">
         <v>119</v>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>Negro</t>
         </is>
       </c>
-      <c r="T3" t="n">
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>#12100E</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Única</t>
+        </is>
+      </c>
+      <c r="AD3" t="n">
         <v>119</v>
       </c>
     </row>
@@ -712,17 +880,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>CATEGORÍAS</t>
         </is>
@@ -772,7 +940,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>MARCAS (línea)</t>
         </is>
@@ -842,9 +1010,9 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>COLORES DE LANZAMIENTO</t>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>VARIANTES = color + talla</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -855,7 +1023,7 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Negro · Espresso (Noé)</t>
+          <t>variacion_N: nombre del color (Negro, Espresso, Beige...)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -865,19 +1033,29 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Beige · Espresso · Negro (Olivia)</t>
+          <t>color_hex_N: color del swatch en hexadecimal, ej. #12100E</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>talla_N: talla de ESA variante (Midi, Full, Única...)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+    </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>NOTAS</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>precio_variacion_N: precio de ESA combinación color + talla</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
     </row>
@@ -885,29 +1063,19 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Obligatorios: nombre, precio, categoria (o categoria_id), marca (o marca_id).</t>
+          <t>Mismo color en otra talla = otra columna de variación.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Puedes usar el nombre de la categoría/marca en vez del ID.</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>activo: si/no · beneficios: separa con comas · variaciones: nombre del color + precio.</t>
-        </is>
-      </c>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>CAMPOS EDITORIALES (ficha del producto)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
     </row>
@@ -915,11 +1083,81 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Las fotos se agregan después desde cada producto en el admin.</t>
+          <t>beneficios / usos_comunes / tallas: valores separados por comas.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>combina_con: IDs de productos separados por coma (ej. 3, 5).</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>instagram: posts separados por ; — cada uno url o url|imagen.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>NOTAS</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Obligatorios: nombre, precio, categoria (o categoria_id), marca (o marca_id).</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Puedes usar el nombre de la categoría/marca en vez del ID.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>activo: si/no · color_hex es opcional pero recomendado.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Las fotos se agregan después desde cada producto en el admin.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>